<commit_message>
Generate full-fidelity clean workbooks with source-parity totals
</commit_message>
<xml_diff>
--- a/clean-import-workbooks/Business_Workbook_Clean_2025.xlsx
+++ b/clean-import-workbooks/Business_Workbook_Clean_2025.xlsx
@@ -905,7 +905,7 @@
         <v>1260000</v>
       </c>
       <c r="C2" s="1">
-        <v>46110.93764182871</v>
+        <v>46110.9546134375</v>
       </c>
       <c r="E2" t="str">
         <v>other</v>
@@ -919,7 +919,7 @@
         <v>329500</v>
       </c>
       <c r="C3" s="1">
-        <v>46110.937641840275</v>
+        <v>46110.9546134375</v>
       </c>
       <c r="E3" t="str">
         <v>other</v>
@@ -933,7 +933,7 @@
         <v>70000</v>
       </c>
       <c r="C4" s="1">
-        <v>46110.937641840275</v>
+        <v>46110.9546134375</v>
       </c>
       <c r="E4" t="str">
         <v>other</v>
@@ -947,7 +947,7 @@
         <v>200000</v>
       </c>
       <c r="C5" s="1">
-        <v>46110.937641840275</v>
+        <v>46110.9546134375</v>
       </c>
       <c r="E5" t="str">
         <v>other</v>
@@ -961,7 +961,7 @@
         <v>59500</v>
       </c>
       <c r="C6" s="1">
-        <v>46110.93764185185</v>
+        <v>46110.9546134375</v>
       </c>
       <c r="E6" t="str">
         <v>other</v>

</xml_diff>